<commit_message>
Sumar 5 nuevos pliegos para dar cuenta (PE-300 a PE-304/26)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Acuerdos_gestion_Milei.xlsx
+++ b/Acuerdos_gestion_Milei.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V224"/>
+  <dimension ref="A1:V229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18584,6 +18584,131 @@
         </is>
       </c>
     </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B225">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/304.26/PE/AC","304")</f>
+        <v/>
+      </c>
+      <c r="C225">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/304.26/PE/AC","2026")</f>
+        <v/>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 273/26 QUE SOLICITA ACUERDO PARA DESIGNAR JUEZ PENAL FEDERAL DEL JUZGADO FEDERAL DE GARANTIAS CON ASIENTO EN LA CDAD. DE RAFAELA, PROV. DE SANTA FE, AL DR. GUIDO YERCOVICH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B226">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/303.26/PE/AC","303")</f>
+        <v/>
+      </c>
+      <c r="C226">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/303.26/PE/AC","2026")</f>
+        <v/>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 272/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES DEL TRABAJO DE LA CAPITAL FEDERAL, SALA VIII, A LA DRA. ROSALIA ROMERO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B227">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/302.26/PE/AC","302")</f>
+        <v/>
+      </c>
+      <c r="C227">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/302.26/PE/AC","2026")</f>
+        <v/>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 271/26 QUE SOLICITA ACUERDO PARA DESIGNAR JUEZ DE CAMARA DEL TRIBUNAL ORAL EN LO CRIMINAL Y CORRECCIONAL N° 26 DE LA CAPITAL FEDERAL, AL DR. EDUARDO ANIBAL AGUAYO.</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B228">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/301.26/PE/AC","301")</f>
+        <v/>
+      </c>
+      <c r="C228">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/301.26/PE/AC","2026")</f>
+        <v/>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 270/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO CIVIL Y COMERCIAL FEDERAL DE LA CAPITAL FEDERAL, SALA III, AL DR. CAMILO JORGE ALMEIDA PONS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B229">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/300.26/PE/AC","300")</f>
+        <v/>
+      </c>
+      <c r="C229">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/300.26/PE/AC","2026")</f>
+        <v/>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 269/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO CIVIL Y COMERCIAL FEDERAL DE LA CAPITAL FEDERAL SALA II, AL DR. ALEJANDRO JORGE NOBILI.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizar trazabilidad al 28/10: PE-277 a 304 dados cuenta el 17/09 y sumar PE-308 a 312
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Acuerdos_gestion_Milei.xlsx
+++ b/Acuerdos_gestion_Milei.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V229"/>
+  <dimension ref="A1:V234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -555,7 +555,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -700,7 +700,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -1282,7 +1282,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 29  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 28  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 28  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1571,7 +1571,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 28  -</t>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -18608,6 +18608,39 @@
           <t>MENSAJE N° 273/26 QUE SOLICITA ACUERDO PARA DESIGNAR JUEZ PENAL FEDERAL DEL JUZGADO FEDERAL DE GARANTIAS CON ASIENTO EN LA CDAD. DE RAFAELA, PROV. DE SANTA FE, AL DR. GUIDO YERCOVICH.</t>
         </is>
       </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
+        </is>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11/09/2026 -</t>
+        </is>
+      </c>
+      <c r="L225" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -</t>
+        </is>
+      </c>
+      <c r="M225" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11/09/2026 -</t>
+        </is>
+      </c>
+      <c r="N225" t="n">
+        <v>71</v>
+      </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS</t>
+        </is>
+      </c>
+      <c r="P225" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -18633,6 +18666,39 @@
           <t>MENSAJE N° 272/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES DEL TRABAJO DE LA CAPITAL FEDERAL, SALA VIII, A LA DRA. ROSALIA ROMERO.</t>
         </is>
       </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
+        </is>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11/09/2026 -</t>
+        </is>
+      </c>
+      <c r="L226" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -</t>
+        </is>
+      </c>
+      <c r="M226" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11/09/2026 -</t>
+        </is>
+      </c>
+      <c r="N226" t="n">
+        <v>71</v>
+      </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS</t>
+        </is>
+      </c>
+      <c r="P226" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -18658,6 +18724,39 @@
           <t>MENSAJE N° 271/26 QUE SOLICITA ACUERDO PARA DESIGNAR JUEZ DE CAMARA DEL TRIBUNAL ORAL EN LO CRIMINAL Y CORRECCIONAL N° 26 DE LA CAPITAL FEDERAL, AL DR. EDUARDO ANIBAL AGUAYO.</t>
         </is>
       </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
+        </is>
+      </c>
+      <c r="J227" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11/09/2026 -</t>
+        </is>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -</t>
+        </is>
+      </c>
+      <c r="M227" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11/09/2026 -</t>
+        </is>
+      </c>
+      <c r="N227" t="n">
+        <v>71</v>
+      </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS</t>
+        </is>
+      </c>
+      <c r="P227" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -18683,6 +18782,39 @@
           <t>MENSAJE N° 270/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO CIVIL Y COMERCIAL FEDERAL DE LA CAPITAL FEDERAL, SALA III, AL DR. CAMILO JORGE ALMEIDA PONS.</t>
         </is>
       </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
+        </is>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11/09/2026 -</t>
+        </is>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -</t>
+        </is>
+      </c>
+      <c r="M228" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11/09/2026 -</t>
+        </is>
+      </c>
+      <c r="N228" t="n">
+        <v>71</v>
+      </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS</t>
+        </is>
+      </c>
+      <c r="P228" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -18706,6 +18838,329 @@
       <c r="E229" t="inlineStr">
         <is>
           <t>MENSAJE N° 269/26 QUE SOLICITA ACUERDO PARA DESIGNAR VOCAL DE LA CAMARA NACIONAL DE APELACIONES EN LO CIVIL Y COMERCIAL FEDERAL DE LA CAPITAL FEDERAL SALA II, AL DR. ALEJANDRO JORGE NOBILI.</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 30 17/09/2026 -</t>
+        </is>
+      </c>
+      <c r="J229" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11/09/2026 -</t>
+        </is>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -</t>
+        </is>
+      </c>
+      <c r="M229" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11/09/2026 -</t>
+        </is>
+      </c>
+      <c r="N229" t="n">
+        <v>71</v>
+      </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS</t>
+        </is>
+      </c>
+      <c r="P229" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B230">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/312.26/PE/AC","312")</f>
+        <v/>
+      </c>
+      <c r="C230">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/312.26/PE/AC","2026")</f>
+        <v/>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 280/26 QUE SOLICITA ACUERDO PARA DESIGNAR FISCAL FEDERAL DE LA UNIDAD FISCAL MENDOZA, PROVINCIA DE MENDOZA, AL DR. PABLO GARCIARENA.</t>
+        </is>
+      </c>
+      <c r="G230" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 31  -</t>
+        </is>
+      </c>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 28/09/2026 -</t>
+        </is>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -</t>
+        </is>
+      </c>
+      <c r="M230" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 28/09/2026 -</t>
+        </is>
+      </c>
+      <c r="N230" t="n">
+        <v>71</v>
+      </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS</t>
+        </is>
+      </c>
+      <c r="P230" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B231">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/311.26/PE/AC","311")</f>
+        <v/>
+      </c>
+      <c r="C231">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/311.26/PE/AC","2026")</f>
+        <v/>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 279/26 QUE SOLICITA ACUERDO PARA DESIGNAR JUEZA DE CAMARA DEL TRIBUNAL ORAL EN LO CRIMINAL Y CORRECCIONAL N° 22 DE LA CAPITAL FEDERAL, A LA DRA. LAURA BELLOQUI.</t>
+        </is>
+      </c>
+      <c r="G231" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 31  -</t>
+        </is>
+      </c>
+      <c r="J231" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 28/09/2026 -</t>
+        </is>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -</t>
+        </is>
+      </c>
+      <c r="M231" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 28/09/2026 -</t>
+        </is>
+      </c>
+      <c r="N231" t="n">
+        <v>71</v>
+      </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS</t>
+        </is>
+      </c>
+      <c r="P231" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B232">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/310.26/PE/AC","310")</f>
+        <v/>
+      </c>
+      <c r="C232">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/310.26/PE/AC","2026")</f>
+        <v/>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 278/26 QUE SOLICITA ACUERDO PARA DESIGNAR JUEZ DEL JUZGADO FEDERAL DE PRIMERA INSTANCIA N° 1 DE CORRIENTES, PROVINCIA DE CORRIENTES, AL DR. JUAN CARLOS VALLEJOS.</t>
+        </is>
+      </c>
+      <c r="G232" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 31  -</t>
+        </is>
+      </c>
+      <c r="J232" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 28/09/2026 -</t>
+        </is>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -</t>
+        </is>
+      </c>
+      <c r="M232" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 28/09/2026 -</t>
+        </is>
+      </c>
+      <c r="N232" t="n">
+        <v>71</v>
+      </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS</t>
+        </is>
+      </c>
+      <c r="P232" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B233">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/309.26/PE/AC","309")</f>
+        <v/>
+      </c>
+      <c r="C233">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/309.26/PE/AC","2026")</f>
+        <v/>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 277/26 QUE SOLICITA ACUERDO PARA DESIGNAR DEFENSORA PUBLICA OFICIAL ANTE LOS JUZGADOS Y CAMARA NACIONAL DE APELACIONES EN LO CIVIL, COMERCIAL Y DEL TRABAJO DE LA CAPITAL FEDERAL, DEFENSORIA N° 4, A LA DRA. ANALIA ISABEL CASCONE.</t>
+        </is>
+      </c>
+      <c r="G233" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 31  -</t>
+        </is>
+      </c>
+      <c r="J233" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 28/09/2026 -</t>
+        </is>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -</t>
+        </is>
+      </c>
+      <c r="M233" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 28/09/2026 -</t>
+        </is>
+      </c>
+      <c r="N233" t="n">
+        <v>71</v>
+      </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS</t>
+        </is>
+      </c>
+      <c r="P233" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>PE</t>
+        </is>
+      </c>
+      <c r="B234">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/308.26/PE/AC","308")</f>
+        <v/>
+      </c>
+      <c r="C234">
+        <f>HYPERLINK("https://www.senado.gob.ar/parlamentario/comisiones/verExp/308.26/PE/AC","2026")</f>
+        <v/>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>AC</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>MENSAJE N° 276/26 QUE SOLICITA ACUERDO PARA DESIGNAR JUEZ DEL JUZGADO FEDERAL DE PRIMERA INSTANCIA N° 1 DE SAN JUAN, PROVINCIA DE SAN JUAN, AL DR. GONZALO LUIS GASSULL.</t>
+        </is>
+      </c>
+      <c r="G234" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 31  -</t>
+        </is>
+      </c>
+      <c r="J234" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 28/09/2026 -</t>
+        </is>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  -</t>
+        </is>
+      </c>
+      <c r="M234" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 28/09/2026 -</t>
+        </is>
+      </c>
+      <c r="N234" t="n">
+        <v>71</v>
+      </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>DE ACUERDOS</t>
+        </is>
+      </c>
+      <c r="P234" t="inlineStr">
+        <is>
+          <t>28/09/2026</t>
         </is>
       </c>
     </row>

</xml_diff>